<commit_message>
Changed spelling error on power budget files
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/PowerBudget.xlsx
+++ b/docs/05-Power-Budget/PowerBudget.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gtfr5\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CC94E2-4457-4E02-A7CF-068CDB36BA9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32634635-CCA1-4A6B-8EE4-B96359494139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -147,9 +147,6 @@
     <t xml:space="preserve"> +9V</t>
   </si>
   <si>
-    <t>Auto-Lock Door Sensor</t>
-  </si>
-  <si>
     <t>Matthew Sanderson, Andrew Imoukhuede, Dylan Vierra-Guillermo, Bryce Weber</t>
   </si>
   <si>
@@ -181,6 +178,9 @@
   </si>
   <si>
     <t>Regulator</t>
+  </si>
+  <si>
+    <t>Smart Door Sensor</t>
   </si>
 </sst>
 </file>
@@ -638,7 +638,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -656,6 +655,7 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1044,13 +1044,13 @@
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="54" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="55"/>
+      <c r="B3" s="61" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="54"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="54"/>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
     </row>
@@ -1058,13 +1058,13 @@
       <c r="A4" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="58" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
+      <c r="B4" s="57" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
     </row>
@@ -1072,13 +1072,13 @@
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="57">
+      <c r="B5" s="56">
         <v>1</v>
       </c>
-      <c r="C5" s="55"/>
-      <c r="D5" s="56"/>
-      <c r="E5" s="56"/>
-      <c r="F5" s="55"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="54"/>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
     </row>
@@ -1101,7 +1101,7 @@
       <c r="F6" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="59" t="s">
+      <c r="G6" s="58" t="s">
         <v>11</v>
       </c>
       <c r="H6" s="43" t="s">
@@ -1111,13 +1111,13 @@
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" s="12">
         <v>1</v>
@@ -1136,13 +1136,13 @@
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
@@ -1161,13 +1161,13 @@
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>36</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>37</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
@@ -1212,7 +1212,7 @@
       <c r="F11" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="G11" s="60" t="s">
+      <c r="G11" s="59" t="s">
         <v>11</v>
       </c>
       <c r="H11" s="26" t="s">
@@ -1222,13 +1222,13 @@
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
@@ -1247,13 +1247,13 @@
     <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" s="12">
         <v>1</v>
@@ -1329,16 +1329,16 @@
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="52" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>36</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>37</v>
       </c>
       <c r="E18" s="12">
         <v>1</v>
@@ -1388,7 +1388,7 @@
       <c r="B21" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C21" s="61" t="s">
+      <c r="C21" s="60" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="27" t="s">
@@ -1400,7 +1400,7 @@
       <c r="F21" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="60" t="s">
+      <c r="G21" s="59" t="s">
         <v>11</v>
       </c>
       <c r="H21" s="26" t="s">
@@ -1448,13 +1448,13 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C24" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>36</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>37</v>
       </c>
       <c r="E24" s="12">
         <v>1</v>

</xml_diff>